<commit_message>
Auto-load .env, fix contact form selectors, add Hainaut data
- common.py: dependency-free .env loader so sender vars load without sourcing
- send_contacts.py: fill message placeholders from env; select the visible
  "Get in touch" button (avoid hidden duplicate); fix success detection to
  match the real "Request successfully sent" confirmation
- scrapimmo.py: parse price from the iw-price JSON attribute (clean values
  instead of the mangled duplicated render)
- add hainaut_private_sellers.xlsx (279 private sellers, 268 contacted)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/liege_private_sellers.xlsx
+++ b/liege_private_sellers.xlsx
@@ -464,6 +464,11 @@
           <t>€450,000450000€</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6690,7 +6695,6 @@
           <t>€462,860*462860€</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>